<commit_message>
symbol added to the library and footprint assigned mosfets are yet to be added
</commit_message>
<xml_diff>
--- a/BOM.xlsx
+++ b/BOM.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Sukul\lipo_Charger\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mohan\Project Files\Kicad\Projects\Lipo_Charger_\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA3CD279-5A53-403E-8093-CBD4C1FAC40D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8CEACD3-C730-40E9-8A1C-929A3BD952C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{D2955EA4-FB51-444F-8EAD-6BEDF091E834}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{D2955EA4-FB51-444F-8EAD-6BEDF091E834}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="51">
   <si>
     <t>BQ25703ARSNR</t>
   </si>
@@ -166,13 +166,25 @@
   </si>
   <si>
     <t>https://robu.in/product/33nf-0805-surface-mount-multilayer-ceramic-capacitor-pack-of-50/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">N-Ch Mosfet </t>
+  </si>
+  <si>
+    <t>https://robu.in/product/nvtfs008n04c-hxy-mosfet-40v-60a-1-n-channel-dfn-8l3x3-mosfets-rohs/</t>
+  </si>
+  <si>
+    <t>NVTFS008N04C-HXY MOSFET-40V 60A 1 N-Channel DFN-8L(3×3) MOSFETs ROHS</t>
+  </si>
+  <si>
+    <t>P-Ch Mosfet</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -187,6 +199,12 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF333E48"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
@@ -216,7 +234,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
@@ -233,6 +251,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -549,16 +570,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DE6D481B-BD3B-435E-941B-4DEA1912EF10}">
-  <dimension ref="A1:E15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:E17"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="25.7109375" customWidth="1"/>
-    <col min="2" max="2" width="15.140625" customWidth="1"/>
-    <col min="3" max="3" width="51.7109375" customWidth="1"/>
-    <col min="4" max="4" width="122.28515625" customWidth="1"/>
+    <col min="1" max="1" width="25.6640625" customWidth="1"/>
+    <col min="2" max="2" width="15.109375" customWidth="1"/>
+    <col min="3" max="3" width="51.6640625" customWidth="1"/>
+    <col min="4" max="4" width="122.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>11</v>
       </c>
@@ -575,7 +596,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="B2" t="s">
         <v>0</v>
       </c>
@@ -589,7 +610,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>14</v>
       </c>
@@ -603,7 +624,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>15</v>
       </c>
@@ -617,7 +638,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="42.75" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A5" s="6" t="s">
         <v>14</v>
       </c>
@@ -631,7 +652,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="42.75" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A6" s="6" t="s">
         <v>14</v>
       </c>
@@ -645,7 +666,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>15</v>
       </c>
@@ -659,7 +680,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>15</v>
       </c>
@@ -673,7 +694,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>15</v>
       </c>
@@ -687,7 +708,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>15</v>
       </c>
@@ -701,7 +722,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>15</v>
       </c>
@@ -715,7 +736,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="12" spans="1:5" ht="42.75" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>14</v>
       </c>
@@ -729,7 +750,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="13" spans="1:5" ht="28.5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:5" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>15</v>
       </c>
@@ -743,7 +764,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>15</v>
       </c>
@@ -757,7 +778,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>15</v>
       </c>
@@ -769,6 +790,22 @@
       </c>
       <c r="D15" s="1" t="s">
         <v>42</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>47</v>
+      </c>
+      <c r="C16" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>50</v>
       </c>
     </row>
   </sheetData>
@@ -787,6 +824,7 @@
     <hyperlink ref="D13" r:id="rId12" xr:uid="{2F02F38B-EAE8-4FED-BA3B-75DB92AD6495}"/>
     <hyperlink ref="D14" r:id="rId13" xr:uid="{EA61D0CE-AF2F-4542-96FE-DD00C3782B89}"/>
     <hyperlink ref="D15" r:id="rId14" xr:uid="{095A3256-4C5C-4830-A33E-5A32BC73039B}"/>
+    <hyperlink ref="D16" r:id="rId15" xr:uid="{1FB0BB75-01C7-49B6-9A15-C1545F70C3A3}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
three r one c balancing circuit dev board has to be done yet
</commit_message>
<xml_diff>
--- a/BOM.xlsx
+++ b/BOM.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mohan\Project Files\Kicad\Projects\Lipo_Charger_\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8CEACD3-C730-40E9-8A1C-929A3BD952C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9983778D-EF3F-4116-843C-36DBBFC5D13B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{D2955EA4-FB51-444F-8EAD-6BEDF091E834}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="62">
   <si>
     <t>BQ25703ARSNR</t>
   </si>
@@ -45,9 +45,6 @@
     <t>link</t>
   </si>
   <si>
-    <t xml:space="preserve">10k ohm </t>
-  </si>
-  <si>
     <t>https://roboticsdna.in/product/10k%cf%89-thick-film-smd-resistor-0805-%c2%b15-tolerence-100-pcs/</t>
   </si>
   <si>
@@ -174,17 +171,54 @@
     <t>https://robu.in/product/nvtfs008n04c-hxy-mosfet-40v-60a-1-n-channel-dfn-8l3x3-mosfets-rohs/</t>
   </si>
   <si>
-    <t>NVTFS008N04C-HXY MOSFET-40V 60A 1 N-Channel DFN-8L(3×3) MOSFETs ROHS</t>
-  </si>
-  <si>
     <t>P-Ch Mosfet</t>
+  </si>
+  <si>
+    <t>https://robu.in/product/dmp3013sfv-hxy-mosfet-30v-55a-1-p-channel-dfn-8l3x3-mosfets-rohs/?gad_source=1&amp;gad_campaignid=17427802703&amp;gbraid=0AAAAADvLFWcc9ic22VFoIsUrmP70-iK2S&amp;gclid=CjwKCAiAqprNBhB6EiwAMe3yhmZg5MkbZV4v0Mz0zXMxZnOSODpvHE6NX8wy7lr8cC_BVq8gRN_WFxoCoDoQAvD_BwE</t>
+  </si>
+  <si>
+    <t>DMP3013SFV-HXY MOSFET-30V 55A 1 P-Channel DFN-8L(3×3) MOSFETs ROHS</t>
+  </si>
+  <si>
+    <t>NVTFS008N04C-HXY MOSFET-40V 60A 1 N-Channel DFN-8L(3×3) MOSFETs ROHS(high power)</t>
+  </si>
+  <si>
+    <t>https://robu.in/product/nx7002akar-nexperia-nx7002akar-power-mosfet-n-channel-60-v-190-ma-3-ohm-to-236ab-surface-mount/</t>
+  </si>
+  <si>
+    <t>NX7002AKAR-NEXPERIA-NX7002AKAR-Power MOSFET, N Channel, 60 V, 190 mA, 3 ohm, TO-236AB, Surface Mount(logic level)</t>
+  </si>
+  <si>
+    <t>n ch</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10k ohm   </t>
+  </si>
+  <si>
+    <t>10ohm</t>
+  </si>
+  <si>
+    <t>https://robu.in/product/rc0603fr-0710rl-yageo-smd-chip-resistor-10-ohm-%C2%B1-1-100-mw-0603-1608-metric-thick-film-general-purpose/?gad_source=1&amp;gad_campaignid=17427802703&amp;gbraid=0AAAAADvLFWcc9ic22VFoIsUrmP70-iK2S&amp;gclid=CjwKCAiAqprNBhB6EiwAMe3yhp2p3iNucUvdWl7XG0jygr1PJz7sX9FLgj0NmdbFsM6PPRNKa5W0FxoCdoMQAvD_BwE</t>
+  </si>
+  <si>
+    <t>RC0603FR-0710RL-Yageo-SMD Chip Resistor, 10 ohm, ± 1%, 100 mW, 0603 [1608 Metric], Thick Film, General Purpose</t>
+  </si>
+  <si>
+    <t>10k</t>
+  </si>
+  <si>
+    <t>STM32F401CCU6 Minimum System Board Microcomputer STM32 ARM Core Board
+Rated 5.00 out of 5 based on 2customer ratings</t>
+  </si>
+  <si>
+    <t>https://robu.in/product/stm32f401ccu6-minimum-system-board-microcomputer-stm32-arm-core-board/?gad_source=1&amp;gad_campaignid=21296336107&amp;gbraid=0AAAAADvLFWcL67koJzc385ab_1M1-pg_p&amp;gclid=Cj0KCQiA8KTNBhD_ARIsAOvp6DILX1pNxbqe0o0_XI9qCElJ-CShK7zQ6NLs64tNfs0p0I6sI0Q6OhIaAirYEALw_wcB</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -199,12 +233,6 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF333E48"/>
-      <name val="Arial"/>
-      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
@@ -252,8 +280,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -570,7 +598,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DE6D481B-BD3B-435E-941B-4DEA1912EF10}">
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E20"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="25.6640625" customWidth="1"/>
@@ -581,7 +609,7 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B1" t="s">
         <v>4</v>
@@ -601,7 +629,7 @@
         <v>0</v>
       </c>
       <c r="C2" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>1</v>
@@ -612,200 +640,239 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>14</v>
-      </c>
-      <c r="B3">
-        <v>10</v>
+        <v>13</v>
+      </c>
+      <c r="B3" t="s">
+        <v>59</v>
       </c>
       <c r="C3" t="s">
+        <v>55</v>
+      </c>
+      <c r="D3" s="1" t="s">
         <v>6</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>7</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C4" t="s">
         <v>8</v>
       </c>
-      <c r="C4" t="s">
+      <c r="D4" s="2" t="s">
         <v>9</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>10</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A5" s="6" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B5" s="6">
         <v>4.99</v>
       </c>
       <c r="C5" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D5" s="5" t="s">
         <v>12</v>
-      </c>
-      <c r="D5" s="5" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A6" s="6" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B6" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B7" t="s">
+        <v>19</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="D7" s="1" t="s">
         <v>20</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>21</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B8" t="s">
+        <v>21</v>
+      </c>
+      <c r="C8" t="s">
+        <v>23</v>
+      </c>
+      <c r="D8" s="1" t="s">
         <v>22</v>
-      </c>
-      <c r="C8" t="s">
-        <v>24</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>23</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B9" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C9" t="s">
+        <v>44</v>
+      </c>
+      <c r="D9" s="1" t="s">
         <v>45</v>
-      </c>
-      <c r="D9" s="1" t="s">
-        <v>46</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B10" t="s">
+        <v>26</v>
+      </c>
+      <c r="C10" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="C10" s="3" t="s">
+      <c r="D10" s="1" t="s">
         <v>28</v>
-      </c>
-      <c r="D10" s="1" t="s">
-        <v>29</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B11" t="s">
+        <v>29</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D11" s="1" t="s">
         <v>30</v>
-      </c>
-      <c r="C11" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="D11" s="1" t="s">
-        <v>31</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B12" t="s">
+        <v>32</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="D12" s="5" t="s">
         <v>33</v>
-      </c>
-      <c r="C12" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="D12" s="5" t="s">
-        <v>34</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B13" t="s">
+        <v>35</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="D13" s="1" t="s">
         <v>36</v>
-      </c>
-      <c r="C13" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="D13" s="1" t="s">
-        <v>37</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B14" t="s">
+        <v>37</v>
+      </c>
+      <c r="C14" t="s">
+        <v>39</v>
+      </c>
+      <c r="D14" s="1" t="s">
         <v>38</v>
-      </c>
-      <c r="C14" t="s">
-        <v>40</v>
-      </c>
-      <c r="D14" s="1" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B15" t="s">
+        <v>40</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="D15" s="1" t="s">
         <v>41</v>
-      </c>
-      <c r="C15" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="D15" s="1" t="s">
-        <v>42</v>
       </c>
     </row>
     <row r="16" spans="1:5" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
+        <v>46</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="D16" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="C16" s="7" t="s">
+    </row>
+    <row r="17" spans="1:4" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>48</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="D17" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="D16" s="1" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A17" t="s">
-        <v>50</v>
+    </row>
+    <row r="18" spans="1:4" ht="41.4" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>54</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" ht="41.4" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>13</v>
+      </c>
+      <c r="B19" t="s">
+        <v>56</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="C20" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="D20" s="5" t="s">
+        <v>61</v>
       </c>
     </row>
   </sheetData>
@@ -825,6 +892,10 @@
     <hyperlink ref="D14" r:id="rId13" xr:uid="{EA61D0CE-AF2F-4542-96FE-DD00C3782B89}"/>
     <hyperlink ref="D15" r:id="rId14" xr:uid="{095A3256-4C5C-4830-A33E-5A32BC73039B}"/>
     <hyperlink ref="D16" r:id="rId15" xr:uid="{1FB0BB75-01C7-49B6-9A15-C1545F70C3A3}"/>
+    <hyperlink ref="D17" r:id="rId16" display="https://robu.in/product/dmp3013sfv-hxy-mosfet-30v-55a-1-p-channel-dfn-8l3x3-mosfets-rohs/?gad_source=1&amp;gad_campaignid=17427802703&amp;gbraid=0AAAAADvLFWcc9ic22VFoIsUrmP70-iK2S&amp;gclid=CjwKCAiAqprNBhB6EiwAMe3yhmZg5MkbZV4v0Mz0zXMxZnOSODpvHE6NX8wy7lr8cC_BVq8gRN_WFxoCoDoQAvD_BwE" xr:uid="{78AD2645-F0B7-4584-B16E-B5C078037B91}"/>
+    <hyperlink ref="D18" r:id="rId17" xr:uid="{A65B9C57-EAE8-4404-9B21-5D5302B2D9FF}"/>
+    <hyperlink ref="D19" r:id="rId18" display="https://robu.in/product/rc0603fr-0710rl-yageo-smd-chip-resistor-10-ohm-%C2%B1-1-100-mw-0603-1608-metric-thick-film-general-purpose/?gad_source=1&amp;gad_campaignid=17427802703&amp;gbraid=0AAAAADvLFWcc9ic22VFoIsUrmP70-iK2S&amp;gclid=CjwKCAiAqprNBhB6EiwAMe3yhp2p3iNucUvdWl7XG0jygr1PJz7sX9FLgj0NmdbFsM6PPRNKa5W0FxoCdoMQAvD_BwE" xr:uid="{D88A1E0A-3DFC-4A4B-8A9B-A6BA36D029FF}"/>
+    <hyperlink ref="D20" r:id="rId19" display="https://robu.in/product/stm32f401ccu6-minimum-system-board-microcomputer-stm32-arm-core-board/?gad_source=1&amp;gad_campaignid=21296336107&amp;gbraid=0AAAAADvLFWcL67koJzc385ab_1M1-pg_p&amp;gclid=Cj0KCQiA8KTNBhD_ARIsAOvp6DILX1pNxbqe0o0_XI9qCElJ-CShK7zQ6NLs64tNfs0p0I6sI0Q6OhIaAirYEALw_wcB" xr:uid="{D94015E3-7EBA-4922-BEBD-00810B7445B6}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
adcc has to be done stm dev board if needed has to be inccluded
</commit_message>
<xml_diff>
--- a/BOM.xlsx
+++ b/BOM.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mohan\Project Files\Kicad\Projects\Lipo_Charger_\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9983778D-EF3F-4116-843C-36DBBFC5D13B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78FD34D8-7BA3-4E7D-A67E-C61E01996823}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{D2955EA4-FB51-444F-8EAD-6BEDF091E834}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="68">
   <si>
     <t>BQ25703ARSNR</t>
   </si>
@@ -212,6 +212,24 @@
   </si>
   <si>
     <t>https://robu.in/product/stm32f401ccu6-minimum-system-board-microcomputer-stm32-arm-core-board/?gad_source=1&amp;gad_campaignid=21296336107&amp;gbraid=0AAAAADvLFWcL67koJzc385ab_1M1-pg_p&amp;gclid=Cj0KCQiA8KTNBhD_ARIsAOvp6DILX1pNxbqe0o0_XI9qCElJ-CShK7zQ6NLs64tNfs0p0I6sI0Q6OhIaAirYEALw_wcB</t>
+  </si>
+  <si>
+    <t>1800pf</t>
+  </si>
+  <si>
+    <t>https://robu.in/product/1-8nf-1800pf-50v-capacitor-0805-smd-package-pack-of-30/</t>
+  </si>
+  <si>
+    <t>1.8nF (1800pF) 50V Capacitor – 0805 SMD Package</t>
+  </si>
+  <si>
+    <t>0.010hm</t>
+  </si>
+  <si>
+    <t>https://robu.in/product/0-01-ohm-3w-surface-mount-sense-resistor-pack-of-3/#tab-specification</t>
+  </si>
+  <si>
+    <t>0.01 Ohm 3W SMD2512 Surface Mount Sense Resistor</t>
   </si>
 </sst>
 </file>
@@ -598,7 +616,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DE6D481B-BD3B-435E-941B-4DEA1912EF10}">
-  <dimension ref="A1:E20"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="25.6640625" customWidth="1"/>
@@ -873,6 +891,31 @@
       </c>
       <c r="D20" s="5" t="s">
         <v>61</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>14</v>
+      </c>
+      <c r="B21" t="s">
+        <v>62</v>
+      </c>
+      <c r="C21" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="D21" s="1" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B22" t="s">
+        <v>65</v>
+      </c>
+      <c r="C22" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="D22" s="1" t="s">
+        <v>66</v>
       </c>
     </row>
   </sheetData>
@@ -896,6 +939,8 @@
     <hyperlink ref="D18" r:id="rId17" xr:uid="{A65B9C57-EAE8-4404-9B21-5D5302B2D9FF}"/>
     <hyperlink ref="D19" r:id="rId18" display="https://robu.in/product/rc0603fr-0710rl-yageo-smd-chip-resistor-10-ohm-%C2%B1-1-100-mw-0603-1608-metric-thick-film-general-purpose/?gad_source=1&amp;gad_campaignid=17427802703&amp;gbraid=0AAAAADvLFWcc9ic22VFoIsUrmP70-iK2S&amp;gclid=CjwKCAiAqprNBhB6EiwAMe3yhp2p3iNucUvdWl7XG0jygr1PJz7sX9FLgj0NmdbFsM6PPRNKa5W0FxoCdoMQAvD_BwE" xr:uid="{D88A1E0A-3DFC-4A4B-8A9B-A6BA36D029FF}"/>
     <hyperlink ref="D20" r:id="rId19" display="https://robu.in/product/stm32f401ccu6-minimum-system-board-microcomputer-stm32-arm-core-board/?gad_source=1&amp;gad_campaignid=21296336107&amp;gbraid=0AAAAADvLFWcL67koJzc385ab_1M1-pg_p&amp;gclid=Cj0KCQiA8KTNBhD_ARIsAOvp6DILX1pNxbqe0o0_XI9qCElJ-CShK7zQ6NLs64tNfs0p0I6sI0Q6OhIaAirYEALw_wcB" xr:uid="{D94015E3-7EBA-4922-BEBD-00810B7445B6}"/>
+    <hyperlink ref="D21" r:id="rId20" xr:uid="{5F2CC437-E6F2-42D3-BD67-7C56BD6EC2EB}"/>
+    <hyperlink ref="D22" r:id="rId21" location="tab-specification" xr:uid="{4918E632-35B3-43E5-BEDC-5262083A5839}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
need to checked sch and then routing thickness has to be calculated and ground fill has to be added
</commit_message>
<xml_diff>
--- a/BOM.xlsx
+++ b/BOM.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mohan\Project Files\Kicad\Projects\Lipo_Charger_\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78FD34D8-7BA3-4E7D-A67E-C61E01996823}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B585F03-E5E9-449A-B981-903D8CBC5C23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{D2955EA4-FB51-444F-8EAD-6BEDF091E834}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="80">
   <si>
     <t>BQ25703ARSNR</t>
   </si>
@@ -230,6 +230,42 @@
   </si>
   <si>
     <t>0.01 Ohm 3W SMD2512 Surface Mount Sense Resistor</t>
+  </si>
+  <si>
+    <t>https://robu.in/product/cs3216x7r225k500nri-samwha-50v-2-2uf-x7r-%C2%B110-1206-multilayer-ceramic-capacitors-mlcc-smd-smt-rohs/?gad_source=1&amp;gad_campaignid=17427802703&amp;gbraid=0AAAAADvLFWez-4uIsPU8kN7QaZXojl8Nx&amp;gclid=Cj0KCQiAk6rNBhCxARIsAN5mQLu4P3mbwqSfoiOgoZc18y9ors1pnUlGGtfe9OsnrAWCB2ogXfLDYasaAueUEALw_wcB#tab-specification</t>
+  </si>
+  <si>
+    <t>2.2uf</t>
+  </si>
+  <si>
+    <t>3.3k</t>
+  </si>
+  <si>
+    <t>https://robu.in/product/ac0603fr-0739kl-yageo-res-thick-film-0603-39k-ohm-1-0-1w1-10w-%C2%B1100ppm-c-pad-smd-t-r-automotive-aec-q200/?utm_source=chatgpt.com</t>
+  </si>
+  <si>
+    <t>https://robu.in/product/ac0805fr-078k2l-yageo-res-thick-film-0805-8-2k-ohm-1-0-125w1-8w-%c2%b1100ppm-c-pad-smd-t-r-automotive-aec-q200/</t>
+  </si>
+  <si>
+    <t>8.2k</t>
+  </si>
+  <si>
+    <t>39k</t>
+  </si>
+  <si>
+    <t>https://robu.in/product/ac0603fr-0727kl-yageo-res-thick-film-0603-27k-ohm-1-0-1w1-10w-%c2%b1100ppm-c-pad-smd-t-r-automotive-aec-q200/</t>
+  </si>
+  <si>
+    <t>27k</t>
+  </si>
+  <si>
+    <t>15k</t>
+  </si>
+  <si>
+    <t>https://robu.in/product/ac0603fr-0715kl-yageo-res-thick-film-0603-15k-ohm-1-0-1w1-10w-%c2%b1100ppm-c-pad-smd-t-r-automotive-aec-q200/</t>
+  </si>
+  <si>
+    <t>https://robu.in/product/3-3k-ohm-1-4w-0603-surface-mount-chip-resistor-pack-of-100/</t>
   </si>
 </sst>
 </file>
@@ -616,7 +652,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DE6D481B-BD3B-435E-941B-4DEA1912EF10}">
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:E28"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="25.6640625" customWidth="1"/>
@@ -908,6 +944,9 @@
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>13</v>
+      </c>
       <c r="B22" t="s">
         <v>65</v>
       </c>
@@ -916,6 +955,72 @@
       </c>
       <c r="D22" s="1" t="s">
         <v>66</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>14</v>
+      </c>
+      <c r="B23" t="s">
+        <v>69</v>
+      </c>
+      <c r="D23" s="1" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>13</v>
+      </c>
+      <c r="B24" t="s">
+        <v>74</v>
+      </c>
+      <c r="D24" s="1" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
+        <v>13</v>
+      </c>
+      <c r="B25" t="s">
+        <v>73</v>
+      </c>
+      <c r="D25" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
+        <v>13</v>
+      </c>
+      <c r="B26" t="s">
+        <v>76</v>
+      </c>
+      <c r="D26" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A27" t="s">
+        <v>13</v>
+      </c>
+      <c r="B27" t="s">
+        <v>77</v>
+      </c>
+      <c r="D27" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
+        <v>13</v>
+      </c>
+      <c r="B28" t="s">
+        <v>70</v>
+      </c>
+      <c r="D28" t="s">
+        <v>79</v>
       </c>
     </row>
   </sheetData>
@@ -941,6 +1046,8 @@
     <hyperlink ref="D20" r:id="rId19" display="https://robu.in/product/stm32f401ccu6-minimum-system-board-microcomputer-stm32-arm-core-board/?gad_source=1&amp;gad_campaignid=21296336107&amp;gbraid=0AAAAADvLFWcL67koJzc385ab_1M1-pg_p&amp;gclid=Cj0KCQiA8KTNBhD_ARIsAOvp6DILX1pNxbqe0o0_XI9qCElJ-CShK7zQ6NLs64tNfs0p0I6sI0Q6OhIaAirYEALw_wcB" xr:uid="{D94015E3-7EBA-4922-BEBD-00810B7445B6}"/>
     <hyperlink ref="D21" r:id="rId20" xr:uid="{5F2CC437-E6F2-42D3-BD67-7C56BD6EC2EB}"/>
     <hyperlink ref="D22" r:id="rId21" location="tab-specification" xr:uid="{4918E632-35B3-43E5-BEDC-5262083A5839}"/>
+    <hyperlink ref="D23" r:id="rId22" location="tab-specification" display="https://robu.in/product/cs3216x7r225k500nri-samwha-50v-2-2uf-x7r-%C2%B110-1206-multilayer-ceramic-capacitors-mlcc-smd-smt-rohs/?gad_source=1&amp;gad_campaignid=17427802703&amp;gbraid=0AAAAADvLFWez-4uIsPU8kN7QaZXojl8Nx&amp;gclid=Cj0KCQiAk6rNBhCxARIsAN5mQLu4P3mbwqSfoiOgoZc18y9ors1pnUlGGtfe9OsnrAWCB2ogXfLDYasaAueUEALw_wcB#tab-specification" xr:uid="{ACCB9BF8-C2CC-4FD9-9324-72D8C0F29D8B}"/>
+    <hyperlink ref="D24" r:id="rId23" xr:uid="{5FA77FDF-E360-4145-AAF8-A6F4251BFF13}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
need to add stm dev boarrd and silkscreen managing sch rechecik and trace width check eed to add gnd and power plane
</commit_message>
<xml_diff>
--- a/BOM.xlsx
+++ b/BOM.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mohan\Project Files\Kicad\Projects\Lipo_Charger_\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B585F03-E5E9-449A-B981-903D8CBC5C23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35EE981A-6C04-435C-A682-D45F588C66EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{D2955EA4-FB51-444F-8EAD-6BEDF091E834}"/>
   </bookViews>
@@ -244,9 +244,6 @@
     <t>https://robu.in/product/ac0603fr-0739kl-yageo-res-thick-film-0603-39k-ohm-1-0-1w1-10w-%C2%B1100ppm-c-pad-smd-t-r-automotive-aec-q200/?utm_source=chatgpt.com</t>
   </si>
   <si>
-    <t>https://robu.in/product/ac0805fr-078k2l-yageo-res-thick-film-0805-8-2k-ohm-1-0-125w1-8w-%c2%b1100ppm-c-pad-smd-t-r-automotive-aec-q200/</t>
-  </si>
-  <si>
     <t>8.2k</t>
   </si>
   <si>
@@ -266,6 +263,9 @@
   </si>
   <si>
     <t>https://robu.in/product/3-3k-ohm-1-4w-0603-surface-mount-chip-resistor-pack-of-100/</t>
+  </si>
+  <si>
+    <t>https://robu.in/product/rc0603fr-078k2l-yageo-res-thick-film-0603-8-2k-ohm-1-0-1w1-10w-%c2%b1100ppm-c-pad-smd-t-r/</t>
   </si>
 </sst>
 </file>
@@ -973,7 +973,7 @@
         <v>13</v>
       </c>
       <c r="B24" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D24" s="1" t="s">
         <v>71</v>
@@ -984,10 +984,10 @@
         <v>13</v>
       </c>
       <c r="B25" t="s">
-        <v>73</v>
-      </c>
-      <c r="D25" t="s">
         <v>72</v>
+      </c>
+      <c r="D25" s="1" t="s">
+        <v>79</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.3">
@@ -995,10 +995,10 @@
         <v>13</v>
       </c>
       <c r="B26" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D26" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.3">
@@ -1006,10 +1006,10 @@
         <v>13</v>
       </c>
       <c r="B27" t="s">
+        <v>76</v>
+      </c>
+      <c r="D27" t="s">
         <v>77</v>
-      </c>
-      <c r="D27" t="s">
-        <v>78</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.3">
@@ -1020,7 +1020,7 @@
         <v>70</v>
       </c>
       <c r="D28" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
   </sheetData>
@@ -1048,6 +1048,7 @@
     <hyperlink ref="D22" r:id="rId21" location="tab-specification" xr:uid="{4918E632-35B3-43E5-BEDC-5262083A5839}"/>
     <hyperlink ref="D23" r:id="rId22" location="tab-specification" display="https://robu.in/product/cs3216x7r225k500nri-samwha-50v-2-2uf-x7r-%C2%B110-1206-multilayer-ceramic-capacitors-mlcc-smd-smt-rohs/?gad_source=1&amp;gad_campaignid=17427802703&amp;gbraid=0AAAAADvLFWez-4uIsPU8kN7QaZXojl8Nx&amp;gclid=Cj0KCQiAk6rNBhCxARIsAN5mQLu4P3mbwqSfoiOgoZc18y9ors1pnUlGGtfe9OsnrAWCB2ogXfLDYasaAueUEALw_wcB#tab-specification" xr:uid="{ACCB9BF8-C2CC-4FD9-9324-72D8C0F29D8B}"/>
     <hyperlink ref="D24" r:id="rId23" xr:uid="{5FA77FDF-E360-4145-AAF8-A6F4251BFF13}"/>
+    <hyperlink ref="D25" r:id="rId24" xr:uid="{32DAF433-9403-4279-9C7F-090B548FA8BF}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
all the links of the components has been assigned in the library for routing components placement is optimizes need routing
</commit_message>
<xml_diff>
--- a/BOM.xlsx
+++ b/BOM.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mohan\Project Files\Kicad\Projects\Lipo_Charger_\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35EE981A-6C04-435C-A682-D45F588C66EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1DC2A1CB-9450-42FE-8DC6-7EC2B48822D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{D2955EA4-FB51-444F-8EAD-6BEDF091E834}"/>
+    <workbookView xWindow="3675" yWindow="-11640" windowWidth="20730" windowHeight="11760" xr2:uid="{D2955EA4-FB51-444F-8EAD-6BEDF091E834}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="88">
   <si>
     <t>BQ25703ARSNR</t>
   </si>
@@ -43,9 +43,6 @@
   </si>
   <si>
     <t>link</t>
-  </si>
-  <si>
-    <t>https://roboticsdna.in/product/10k%cf%89-thick-film-smd-resistor-0805-%c2%b15-tolerence-100-pcs/</t>
   </si>
   <si>
     <t>10uf</t>
@@ -266,13 +263,40 @@
   </si>
   <si>
     <t>https://robu.in/product/rc0603fr-078k2l-yageo-res-thick-film-0603-8-2k-ohm-1-0-1w1-10w-%c2%b1100ppm-c-pad-smd-t-r/</t>
+  </si>
+  <si>
+    <t>https://robu.in/product/amass-xt60pw30-male-connector-xt60pw-m-g-y/?gad_source=1&amp;gad_campaignid=17427802559&amp;gbraid=0AAAAADvLFWfhks-89lNOnM8tQ5m3yghtb&amp;gclid=CjwKCAjwpcTNBhA5EiwAdO1S9p18uyCkBZMZdjxAzY0inTrlFEcon7oAEEV3vYgDTjTrNs7sAUoaBxoCabEQAvD_BwE</t>
+  </si>
+  <si>
+    <t>xt60 right angled</t>
+  </si>
+  <si>
+    <t xml:space="preserve">47ohm </t>
+  </si>
+  <si>
+    <t>https://roboticsdna.in/product/10k%cf%89-thick-film-smd-resistor-0805-%c2%b     15-tolerence-100-pcs/</t>
+  </si>
+  <si>
+    <t>https://robu.in/product/rc2512jk-0747rl-yageo-smd-chip-resistor-47-ohm-%C2%B1-5-1-w-2512-6432-metric-thick-film-general-purpose/?utm_source=chatgpt.com</t>
+  </si>
+  <si>
+    <t>xt60</t>
+  </si>
+  <si>
+    <t>black pill</t>
+  </si>
+  <si>
+    <t>Inductor 2.2uh</t>
+  </si>
+  <si>
+    <t>https://robu.in/product/cdrh104r-2-2%CE%BCh-power-inductor-pack-of-5/?gad_source=1&amp;gad_campaignid=17427802703&amp;gbraid=0AAAAADvLFWeYd6KQJmaof5AqwX7G6G7RK&amp;gclid=CjwKCAjw687NBhB4EiwAQ645dmHAlDrRVuziQAJbPZqMJFAUlKgMQ-ZthCMAKLuhHOvZczBMktniURoCJv0QAvD_BwE#tab-robu_other_tab</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -652,18 +676,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DE6D481B-BD3B-435E-941B-4DEA1912EF10}">
-  <dimension ref="A1:E28"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:E31"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="25.6640625" customWidth="1"/>
     <col min="2" max="2" width="15.109375" customWidth="1"/>
     <col min="3" max="3" width="51.6640625" customWidth="1"/>
-    <col min="4" max="4" width="122.33203125" customWidth="1"/>
+    <col min="4" max="4" width="128.21875" customWidth="1"/>
+    <col min="5" max="5" width="39.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5">
       <c r="A1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B1" t="s">
         <v>4</v>
@@ -678,377 +703,412 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="B2" t="s">
-        <v>0</v>
-      </c>
-      <c r="C2" t="s">
-        <v>43</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="E2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" ht="41.4">
+      <c r="A2" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2" s="6">
+        <v>4.99</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5">
       <c r="A3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B3" t="s">
+        <v>64</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5">
+      <c r="A4" t="s">
         <v>13</v>
       </c>
-      <c r="B3" t="s">
-        <v>59</v>
-      </c>
-      <c r="C3" t="s">
+      <c r="B4" t="s">
+        <v>28</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5">
+      <c r="A5" t="s">
+        <v>13</v>
+      </c>
+      <c r="B5" t="s">
+        <v>20</v>
+      </c>
+      <c r="C5" t="s">
+        <v>22</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5">
+      <c r="A6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B6" t="s">
+        <v>58</v>
+      </c>
+      <c r="C6" t="s">
+        <v>54</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="41.4">
+      <c r="A7" t="s">
+        <v>12</v>
+      </c>
+      <c r="B7" t="s">
         <v>55</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="C7" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5">
+      <c r="A8" t="s">
+        <v>13</v>
+      </c>
+      <c r="B8" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
+      <c r="C8" t="s">
+        <v>7</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="41.4">
+      <c r="A9" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B9" t="s">
+        <v>16</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="D9" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="B4" t="s">
-        <v>7</v>
-      </c>
-      <c r="C4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" ht="41.4" x14ac:dyDescent="0.3">
-      <c r="A5" s="6" t="s">
+    </row>
+    <row r="10" spans="1:5">
+      <c r="A10" t="s">
+        <v>12</v>
+      </c>
+      <c r="B10" t="s">
+        <v>75</v>
+      </c>
+      <c r="D10" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5">
+      <c r="A11" t="s">
         <v>13</v>
       </c>
-      <c r="B5" s="6">
-        <v>4.99</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="D5" s="5" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" ht="41.4" x14ac:dyDescent="0.3">
-      <c r="A6" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="B6" t="s">
-        <v>17</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="D6" s="5" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>14</v>
-      </c>
-      <c r="B7" t="s">
-        <v>19</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>14</v>
-      </c>
-      <c r="B8" t="s">
-        <v>21</v>
-      </c>
-      <c r="C8" t="s">
-        <v>23</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
-        <v>14</v>
-      </c>
-      <c r="B9" t="s">
-        <v>24</v>
-      </c>
-      <c r="C9" t="s">
-        <v>44</v>
-      </c>
-      <c r="D9" s="1" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
-        <v>14</v>
-      </c>
-      <c r="B10" t="s">
-        <v>26</v>
-      </c>
-      <c r="C10" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="D10" s="1" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
-        <v>14</v>
-      </c>
       <c r="B11" t="s">
-        <v>29</v>
-      </c>
-      <c r="C11" s="3" t="s">
-        <v>31</v>
+        <v>36</v>
+      </c>
+      <c r="C11" t="s">
+        <v>38</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" ht="41.4" x14ac:dyDescent="0.3">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5">
       <c r="A12" t="s">
         <v>13</v>
       </c>
       <c r="B12" t="s">
+        <v>61</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5">
+      <c r="A13" t="s">
+        <v>13</v>
+      </c>
+      <c r="B13" t="s">
+        <v>25</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5">
+      <c r="A14" t="s">
+        <v>13</v>
+      </c>
+      <c r="B14" t="s">
+        <v>68</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5">
+      <c r="A15" t="s">
+        <v>12</v>
+      </c>
+      <c r="B15" t="s">
+        <v>74</v>
+      </c>
+      <c r="D15" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5">
+      <c r="A16" t="s">
+        <v>12</v>
+      </c>
+      <c r="B16" t="s">
+        <v>69</v>
+      </c>
+      <c r="D16" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5">
+      <c r="A17" t="s">
+        <v>13</v>
+      </c>
+      <c r="B17" t="s">
+        <v>23</v>
+      </c>
+      <c r="C17" t="s">
+        <v>43</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" ht="27.6">
+      <c r="A18" t="s">
+        <v>13</v>
+      </c>
+      <c r="B18" t="s">
+        <v>34</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5">
+      <c r="A19" t="s">
+        <v>12</v>
+      </c>
+      <c r="B19" t="s">
+        <v>72</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" ht="41.4">
+      <c r="A20" t="s">
+        <v>12</v>
+      </c>
+      <c r="B20" t="s">
+        <v>31</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="D20" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="C12" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="D12" s="5" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A13" t="s">
-        <v>14</v>
-      </c>
-      <c r="B13" t="s">
-        <v>35</v>
-      </c>
-      <c r="C13" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="D13" s="1" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A14" t="s">
-        <v>14</v>
-      </c>
-      <c r="B14" t="s">
-        <v>37</v>
-      </c>
-      <c r="C14" t="s">
+    </row>
+    <row r="21" spans="1:5">
+      <c r="A21" t="s">
+        <v>13</v>
+      </c>
+      <c r="B21" t="s">
+        <v>18</v>
+      </c>
+      <c r="C21" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="D21" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5">
+      <c r="B22" t="s">
+        <v>81</v>
+      </c>
+      <c r="D22" s="1" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5">
+      <c r="A23" t="s">
+        <v>13</v>
+      </c>
+      <c r="B23" t="s">
         <v>39</v>
       </c>
-      <c r="D14" s="1" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A15" t="s">
-        <v>14</v>
-      </c>
-      <c r="B15" t="s">
+      <c r="C23" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="D23" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="C15" s="3" t="s">
+    </row>
+    <row r="24" spans="1:5">
+      <c r="A24" t="s">
+        <v>12</v>
+      </c>
+      <c r="B24" t="s">
+        <v>71</v>
+      </c>
+      <c r="D24" s="1" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5">
+      <c r="B25" t="s">
+        <v>0</v>
+      </c>
+      <c r="C25" t="s">
         <v>42</v>
       </c>
-      <c r="D15" s="1" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A16" t="s">
+      <c r="D25" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="E25">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5">
+      <c r="A26" t="s">
+        <v>80</v>
+      </c>
+      <c r="B26" t="s">
+        <v>84</v>
+      </c>
+      <c r="D26" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" ht="27.6">
+      <c r="A27" t="s">
+        <v>45</v>
+      </c>
+      <c r="C27" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="D27" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="C16" s="3" t="s">
+    </row>
+    <row r="28" spans="1:5" ht="27.6">
+      <c r="A28" t="s">
+        <v>47</v>
+      </c>
+      <c r="C28" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="D28" s="1" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" ht="41.4">
+      <c r="A29" t="s">
+        <v>53</v>
+      </c>
+      <c r="C29" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="D29" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="D16" s="1" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A17" t="s">
-        <v>48</v>
-      </c>
-      <c r="C17" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="D17" s="1" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" ht="41.4" x14ac:dyDescent="0.3">
-      <c r="A18" t="s">
-        <v>54</v>
-      </c>
-      <c r="C18" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="D18" s="1" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" ht="41.4" x14ac:dyDescent="0.3">
-      <c r="A19" t="s">
-        <v>13</v>
-      </c>
-      <c r="B19" t="s">
-        <v>56</v>
-      </c>
-      <c r="C19" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="D19" s="1" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="C20" s="7" t="s">
+    </row>
+    <row r="30" spans="1:5" ht="43.2">
+      <c r="A30" t="s">
+        <v>85</v>
+      </c>
+      <c r="C30" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="D30" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="D20" s="5" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A21" t="s">
-        <v>14</v>
-      </c>
-      <c r="B21" t="s">
-        <v>62</v>
-      </c>
-      <c r="C21" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="D21" s="1" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A22" t="s">
-        <v>13</v>
-      </c>
-      <c r="B22" t="s">
-        <v>65</v>
-      </c>
-      <c r="C22" s="3" t="s">
-        <v>67</v>
-      </c>
-      <c r="D22" s="1" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A23" t="s">
-        <v>14</v>
-      </c>
-      <c r="B23" t="s">
-        <v>69</v>
-      </c>
-      <c r="D23" s="1" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A24" t="s">
-        <v>13</v>
-      </c>
-      <c r="B24" t="s">
-        <v>73</v>
-      </c>
-      <c r="D24" s="1" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A25" t="s">
-        <v>13</v>
-      </c>
-      <c r="B25" t="s">
-        <v>72</v>
-      </c>
-      <c r="D25" s="1" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A26" t="s">
-        <v>13</v>
-      </c>
-      <c r="B26" t="s">
-        <v>75</v>
-      </c>
-      <c r="D26" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A27" t="s">
-        <v>13</v>
-      </c>
-      <c r="B27" t="s">
-        <v>76</v>
-      </c>
-      <c r="D27" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A28" t="s">
-        <v>13</v>
-      </c>
-      <c r="B28" t="s">
-        <v>70</v>
-      </c>
-      <c r="D28" t="s">
-        <v>78</v>
+    </row>
+    <row r="31" spans="1:5">
+      <c r="A31" t="s">
+        <v>86</v>
+      </c>
+      <c r="D31" s="1" t="s">
+        <v>87</v>
       </c>
     </row>
   </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:E30">
+    <sortCondition ref="B6:B30"/>
+  </sortState>
   <hyperlinks>
-    <hyperlink ref="D2" r:id="rId1" xr:uid="{0A0A9B8C-658D-44DA-BE52-69A30E115791}"/>
-    <hyperlink ref="D3" r:id="rId2" xr:uid="{3179FDAF-70CE-4E0D-9225-73B33EEE9241}"/>
-    <hyperlink ref="D4" r:id="rId3" location="tab-specification" xr:uid="{B851862D-17DB-4E8D-A010-C13B46B9E1FB}"/>
-    <hyperlink ref="D5" r:id="rId4" xr:uid="{3760DCB1-3480-4B6E-B221-2A5B5A3ED3D3}"/>
-    <hyperlink ref="D6" r:id="rId5" display="https://robu.in/product/ac0402fr-07137kl-yageo-res-thick-film-0402-137k-ohm-1-0-063w1-16w-%C2%B1100ppm-c-pad-smd-t-r-automotive-aec-q200/?gad_source=1&amp;gad_campaignid=17427802703&amp;gbraid=0AAAAADvLFWckUsGFRRIu9JENF8k6hQc3U&amp;gclid=CjwKCAiAh5XNBhAAEiwA_Bu8Fb7RvVYpFw6ihaG1wSCJ7habpWXIudxKK5--gi5ni0UQSLs9Cxl79BoCuJcQAvD_BwE" xr:uid="{C7FCBD7F-DC33-40A8-A846-25D687284E89}"/>
-    <hyperlink ref="D8" r:id="rId6" xr:uid="{37E3D571-32C8-478F-B8FE-417A2504880F}"/>
-    <hyperlink ref="D9" r:id="rId7" xr:uid="{65C20F54-94DE-411F-AC72-6E2AE1B4BAC8}"/>
-    <hyperlink ref="D7" r:id="rId8" xr:uid="{F9D3ADBA-9D5D-4B0D-84D6-2036DE86A908}"/>
-    <hyperlink ref="D11" r:id="rId9" xr:uid="{195D9888-4E47-41D9-BE24-A7AC49505096}"/>
-    <hyperlink ref="D10" r:id="rId10" xr:uid="{F507B3D7-3BE7-4EA7-97A5-7125F104FF70}"/>
-    <hyperlink ref="D12" r:id="rId11" xr:uid="{8A7C05A0-EF96-4B72-8650-638AD8600693}"/>
-    <hyperlink ref="D13" r:id="rId12" xr:uid="{2F02F38B-EAE8-4FED-BA3B-75DB92AD6495}"/>
-    <hyperlink ref="D14" r:id="rId13" xr:uid="{EA61D0CE-AF2F-4542-96FE-DD00C3782B89}"/>
-    <hyperlink ref="D15" r:id="rId14" xr:uid="{095A3256-4C5C-4830-A33E-5A32BC73039B}"/>
-    <hyperlink ref="D16" r:id="rId15" xr:uid="{1FB0BB75-01C7-49B6-9A15-C1545F70C3A3}"/>
-    <hyperlink ref="D17" r:id="rId16" display="https://robu.in/product/dmp3013sfv-hxy-mosfet-30v-55a-1-p-channel-dfn-8l3x3-mosfets-rohs/?gad_source=1&amp;gad_campaignid=17427802703&amp;gbraid=0AAAAADvLFWcc9ic22VFoIsUrmP70-iK2S&amp;gclid=CjwKCAiAqprNBhB6EiwAMe3yhmZg5MkbZV4v0Mz0zXMxZnOSODpvHE6NX8wy7lr8cC_BVq8gRN_WFxoCoDoQAvD_BwE" xr:uid="{78AD2645-F0B7-4584-B16E-B5C078037B91}"/>
-    <hyperlink ref="D18" r:id="rId17" xr:uid="{A65B9C57-EAE8-4404-9B21-5D5302B2D9FF}"/>
-    <hyperlink ref="D19" r:id="rId18" display="https://robu.in/product/rc0603fr-0710rl-yageo-smd-chip-resistor-10-ohm-%C2%B1-1-100-mw-0603-1608-metric-thick-film-general-purpose/?gad_source=1&amp;gad_campaignid=17427802703&amp;gbraid=0AAAAADvLFWcc9ic22VFoIsUrmP70-iK2S&amp;gclid=CjwKCAiAqprNBhB6EiwAMe3yhp2p3iNucUvdWl7XG0jygr1PJz7sX9FLgj0NmdbFsM6PPRNKa5W0FxoCdoMQAvD_BwE" xr:uid="{D88A1E0A-3DFC-4A4B-8A9B-A6BA36D029FF}"/>
-    <hyperlink ref="D20" r:id="rId19" display="https://robu.in/product/stm32f401ccu6-minimum-system-board-microcomputer-stm32-arm-core-board/?gad_source=1&amp;gad_campaignid=21296336107&amp;gbraid=0AAAAADvLFWcL67koJzc385ab_1M1-pg_p&amp;gclid=Cj0KCQiA8KTNBhD_ARIsAOvp6DILX1pNxbqe0o0_XI9qCElJ-CShK7zQ6NLs64tNfs0p0I6sI0Q6OhIaAirYEALw_wcB" xr:uid="{D94015E3-7EBA-4922-BEBD-00810B7445B6}"/>
-    <hyperlink ref="D21" r:id="rId20" xr:uid="{5F2CC437-E6F2-42D3-BD67-7C56BD6EC2EB}"/>
-    <hyperlink ref="D22" r:id="rId21" location="tab-specification" xr:uid="{4918E632-35B3-43E5-BEDC-5262083A5839}"/>
-    <hyperlink ref="D23" r:id="rId22" location="tab-specification" display="https://robu.in/product/cs3216x7r225k500nri-samwha-50v-2-2uf-x7r-%C2%B110-1206-multilayer-ceramic-capacitors-mlcc-smd-smt-rohs/?gad_source=1&amp;gad_campaignid=17427802703&amp;gbraid=0AAAAADvLFWez-4uIsPU8kN7QaZXojl8Nx&amp;gclid=Cj0KCQiAk6rNBhCxARIsAN5mQLu4P3mbwqSfoiOgoZc18y9ors1pnUlGGtfe9OsnrAWCB2ogXfLDYasaAueUEALw_wcB#tab-specification" xr:uid="{ACCB9BF8-C2CC-4FD9-9324-72D8C0F29D8B}"/>
-    <hyperlink ref="D24" r:id="rId23" xr:uid="{5FA77FDF-E360-4145-AAF8-A6F4251BFF13}"/>
-    <hyperlink ref="D25" r:id="rId24" xr:uid="{32DAF433-9403-4279-9C7F-090B548FA8BF}"/>
+    <hyperlink ref="D25" r:id="rId1" xr:uid="{0A0A9B8C-658D-44DA-BE52-69A30E115791}"/>
+    <hyperlink ref="D6" r:id="rId2" xr:uid="{3179FDAF-70CE-4E0D-9225-73B33EEE9241}"/>
+    <hyperlink ref="D8" r:id="rId3" location="tab-specification" xr:uid="{B851862D-17DB-4E8D-A010-C13B46B9E1FB}"/>
+    <hyperlink ref="D2" r:id="rId4" xr:uid="{3760DCB1-3480-4B6E-B221-2A5B5A3ED3D3}"/>
+    <hyperlink ref="D9" r:id="rId5" display="https://robu.in/product/ac0402fr-07137kl-yageo-res-thick-film-0402-137k-ohm-1-0-063w1-16w-%C2%B1100ppm-c-pad-smd-t-r-automotive-aec-q200/?gad_source=1&amp;gad_campaignid=17427802703&amp;gbraid=0AAAAADvLFWckUsGFRRIu9JENF8k6hQc3U&amp;gclid=CjwKCAiAh5XNBhAAEiwA_Bu8Fb7RvVYpFw6ihaG1wSCJ7habpWXIudxKK5--gi5ni0UQSLs9Cxl79BoCuJcQAvD_BwE" xr:uid="{C7FCBD7F-DC33-40A8-A846-25D687284E89}"/>
+    <hyperlink ref="D5" r:id="rId6" xr:uid="{37E3D571-32C8-478F-B8FE-417A2504880F}"/>
+    <hyperlink ref="D17" r:id="rId7" xr:uid="{65C20F54-94DE-411F-AC72-6E2AE1B4BAC8}"/>
+    <hyperlink ref="D21" r:id="rId8" xr:uid="{F9D3ADBA-9D5D-4B0D-84D6-2036DE86A908}"/>
+    <hyperlink ref="D4" r:id="rId9" xr:uid="{195D9888-4E47-41D9-BE24-A7AC49505096}"/>
+    <hyperlink ref="D13" r:id="rId10" xr:uid="{F507B3D7-3BE7-4EA7-97A5-7125F104FF70}"/>
+    <hyperlink ref="D20" r:id="rId11" xr:uid="{8A7C05A0-EF96-4B72-8650-638AD8600693}"/>
+    <hyperlink ref="D18" r:id="rId12" xr:uid="{2F02F38B-EAE8-4FED-BA3B-75DB92AD6495}"/>
+    <hyperlink ref="D11" r:id="rId13" xr:uid="{EA61D0CE-AF2F-4542-96FE-DD00C3782B89}"/>
+    <hyperlink ref="D23" r:id="rId14" xr:uid="{095A3256-4C5C-4830-A33E-5A32BC73039B}"/>
+    <hyperlink ref="D27" r:id="rId15" xr:uid="{1FB0BB75-01C7-49B6-9A15-C1545F70C3A3}"/>
+    <hyperlink ref="D28" r:id="rId16" display="https://robu.in/product/dmp3013sfv-hxy-mosfet-30v-55a-1-p-channel-dfn-8l3x3-mosfets-rohs/?gad_source=1&amp;gad_campaignid=17427802703&amp;gbraid=0AAAAADvLFWcc9ic22VFoIsUrmP70-iK2S&amp;gclid=CjwKCAiAqprNBhB6EiwAMe3yhmZg5MkbZV4v0Mz0zXMxZnOSODpvHE6NX8wy7lr8cC_BVq8gRN_WFxoCoDoQAvD_BwE" xr:uid="{78AD2645-F0B7-4584-B16E-B5C078037B91}"/>
+    <hyperlink ref="D29" r:id="rId17" xr:uid="{A65B9C57-EAE8-4404-9B21-5D5302B2D9FF}"/>
+    <hyperlink ref="D7" r:id="rId18" display="https://robu.in/product/rc0603fr-0710rl-yageo-smd-chip-resistor-10-ohm-%C2%B1-1-100-mw-0603-1608-metric-thick-film-general-purpose/?gad_source=1&amp;gad_campaignid=17427802703&amp;gbraid=0AAAAADvLFWcc9ic22VFoIsUrmP70-iK2S&amp;gclid=CjwKCAiAqprNBhB6EiwAMe3yhp2p3iNucUvdWl7XG0jygr1PJz7sX9FLgj0NmdbFsM6PPRNKa5W0FxoCdoMQAvD_BwE" xr:uid="{D88A1E0A-3DFC-4A4B-8A9B-A6BA36D029FF}"/>
+    <hyperlink ref="D30" r:id="rId19" display="https://robu.in/product/stm32f401ccu6-minimum-system-board-microcomputer-stm32-arm-core-board/?gad_source=1&amp;gad_campaignid=21296336107&amp;gbraid=0AAAAADvLFWcL67koJzc385ab_1M1-pg_p&amp;gclid=Cj0KCQiA8KTNBhD_ARIsAOvp6DILX1pNxbqe0o0_XI9qCElJ-CShK7zQ6NLs64tNfs0p0I6sI0Q6OhIaAirYEALw_wcB" xr:uid="{D94015E3-7EBA-4922-BEBD-00810B7445B6}"/>
+    <hyperlink ref="D12" r:id="rId20" xr:uid="{5F2CC437-E6F2-42D3-BD67-7C56BD6EC2EB}"/>
+    <hyperlink ref="D3" r:id="rId21" location="tab-specification" xr:uid="{4918E632-35B3-43E5-BEDC-5262083A5839}"/>
+    <hyperlink ref="D14" r:id="rId22" location="tab-specification" display="https://robu.in/product/cs3216x7r225k500nri-samwha-50v-2-2uf-x7r-%C2%B110-1206-multilayer-ceramic-capacitors-mlcc-smd-smt-rohs/?gad_source=1&amp;gad_campaignid=17427802703&amp;gbraid=0AAAAADvLFWez-4uIsPU8kN7QaZXojl8Nx&amp;gclid=Cj0KCQiAk6rNBhCxARIsAN5mQLu4P3mbwqSfoiOgoZc18y9ors1pnUlGGtfe9OsnrAWCB2ogXfLDYasaAueUEALw_wcB#tab-specification" xr:uid="{ACCB9BF8-C2CC-4FD9-9324-72D8C0F29D8B}"/>
+    <hyperlink ref="D19" r:id="rId23" xr:uid="{5FA77FDF-E360-4145-AAF8-A6F4251BFF13}"/>
+    <hyperlink ref="D24" r:id="rId24" xr:uid="{32DAF433-9403-4279-9C7F-090B548FA8BF}"/>
+    <hyperlink ref="D22" r:id="rId25" xr:uid="{A2769295-2D87-4BD8-8447-4313799729E3}"/>
+    <hyperlink ref="D31" r:id="rId26" location="tab-robu_other_tab" display="https://robu.in/product/cdrh104r-2-2%CE%BCh-power-inductor-pack-of-5/?gad_source=1&amp;gad_campaignid=17427802703&amp;gbraid=0AAAAADvLFWeYd6KQJmaof5AqwX7G6G7RK&amp;gclid=CjwKCAjw687NBhB4EiwAQ645dmHAlDrRVuziQAJbPZqMJFAUlKgMQ-ZthCMAKLuhHOvZczBMktniURoCJv0QAvD_BwE#tab-robu_other_tab" xr:uid="{2599D4D5-D5D8-40CC-89F6-8F96996F6D8C}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>